<commit_message>
feat: change shapes namespace to hrishapes
</commit_message>
<xml_diff>
--- a/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-activity.xlsx
+++ b/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-activity.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -828,6 +828,23 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>http://schema.org/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PREFIX</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>hrishapes</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>http://data.health-ri.nl/core/p2/</t>
         </is>
       </c>
     </row>
@@ -853,7 +870,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>https://w3id.org/health-ri/metadata-vocabulary#aux-ActivityShape</t>
+          <t>http://data.health-ri.nl/core/p2/aux-ActivityShape</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -991,7 +1008,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-14 14:14:50</t>
+          <t>2026-10-14 14:30:39</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -1215,7 +1232,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>hri:ActivityShape</t>
+          <t>hrishapes:ActivityShape</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1265,7 +1282,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>https://w3id.org/health-ri/metadata-vocabulary#ActivityShape</t>
+          <t>http://data.health-ri.nl/core/p2/ActivityShape</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1684,12 +1701,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>hri:ActivityShape/dct:type</t>
+          <t>hrishapes:ActivityShape#dct:type</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hri:ActivityShape</t>
+          <t>hrishapes:ActivityShape</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1742,12 +1759,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>hri:ActivityShape/schema:studyDesign</t>
+          <t>hrishapes:ActivityShape#schema:studyDesign</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hri:ActivityShape</t>
+          <t>hrishapes:ActivityShape</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">

</xml_diff>

<commit_message>
fix: fixes change to hrishapes, adds FDP shapes and validation shape
</commit_message>
<xml_diff>
--- a/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-activity.xlsx
+++ b/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-activity.xlsx
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-14 14:30:39</t>
+          <t>2026-10-19 15:50:04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -1747,7 +1747,7 @@
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
-          <t>dash:URIViewer</t>
+          <t>dash:LabelViewer</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -1805,7 +1805,7 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
-          <t>dash:URIViewer</t>
+          <t>dash:LabelViewer</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">

</xml_diff>

<commit_message>
feat: removes study type, added ICD11/aligned Regex, Table.url & Column.propertyURL range to IRI
</commit_message>
<xml_diff>
--- a/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-activity.xlsx
+++ b/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-activity.xlsx
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-19 15:50:04</t>
+          <t>2026-10-26 13:15:51</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -1271,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1756,64 +1756,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>hrishapes:ActivityShape#schema:studyDesign</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>hrishapes:ActivityShape</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>schema:studyDesign</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>study design</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Specifics about the observational study design.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>sh:IRI</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>dash:LabelViewer</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>dash:URIEditor</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>